<commit_message>
chore: rapikan seluruh dokumen skripsi, PR bimbingan Bu Rina, dan dokumentasi teknis ke dalam folder terstruktur
</commit_message>
<xml_diff>
--- a/hasil_pengujian/PERBANDINGAN_MODEL_LAMA_VS_BARU.xlsx
+++ b/hasil_pengujian/PERBANDINGAN_MODEL_LAMA_VS_BARU.xlsx
@@ -1,22 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A51AB4C0-F707-4F1A-9421-CFC78E6E94BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="15" windowWidth="20730" windowHeight="11760" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="1. Ringkasan Perbandingan" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="2. Hasil Pengujian Dibandingkan" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="3. Delta Fitur (Yang Berubah)" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="4. Kesimpulan" state="visible" r:id="rId7"/>
+    <sheet name="1. Ringkasan Perbandingan" sheetId="1" r:id="rId1"/>
+    <sheet name="2. Hasil Pengujian Dibandingkan" sheetId="2" r:id="rId2"/>
+    <sheet name="3. Delta Fitur (Yang Berubah)" sheetId="3" r:id="rId3"/>
+    <sheet name="4. Kesimpulan" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="239">
   <si>
-    <t xml:space="preserve">TABEL PERBANDINGAN SISTEM INTERV-U
+    <t>TABEL PERBANDINGAN SISTEM INTERV-U
 MODEL LAMA (INTERV-U-main) vs MODEL BARU (INTERV-U edit bu rina)
 Data dari Analisis Kode Nyata — 15 Oktober 2026</t>
   </si>
@@ -24,15 +41,15 @@
     <t>ASPEK</t>
   </si>
   <si>
-    <t xml:space="preserve">MODEL LAMA
+    <t>MODEL LAMA
 (INTERV-U-main)</t>
   </si>
   <si>
-    <t xml:space="preserve">MODEL BARU
+    <t>MODEL BARU
 (INTERV-U — edit bu rina)</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS
+    <t>STATUS
 PERUBAHAN</t>
   </si>
   <si>
@@ -42,11 +59,11 @@
     <t>Nama Folder Proyek</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERV-U-main
+    <t>INTERV-U-main
 (D:\INTERV-U-main)</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERV-U
+    <t>INTERV-U
 (D:\intervyou edit bu rina\INTERV-U)</t>
   </si>
   <si>
@@ -104,18 +121,18 @@
     <t>── B. MODEL AI YANG DIGUNAKAN ──</t>
   </si>
   <si>
-    <t xml:space="preserve">Model Evaluasi
+    <t>Model Evaluasi
 (/api/evaluate)</t>
   </si>
   <si>
     <t>gemini-3-flash-preview</t>
   </si>
   <si>
-    <t xml:space="preserve">Model Coaching Chat
+    <t>Model Coaching Chat
 (/api/coaching action:chat)</t>
   </si>
   <si>
-    <t xml:space="preserve">Model TTS Coaching
+    <t>Model TTS Coaching
 (/api/coaching action:speech)</t>
   </si>
   <si>
@@ -128,59 +145,59 @@
     <t>── C. FRAMEWORK EVALUASI (INTI PERBEDAAN) ──</t>
   </si>
   <si>
-    <t xml:space="preserve">Framework STAR
+    <t>Framework STAR
 (Situation-Task-Action-Result)</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ ADA — per QA, score 0-4,
+    <t>✓ ADA — per QA, score 0-4,
 present (true/false) + evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Framework ConCISE
+    <t>Framework ConCISE
 (5 dimensi clarity/structure)</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ ADA — 5 dimensi skor 1-10,
+    <t>✓ ADA — 5 dimensi skor 1-10,
 total max 50</t>
   </si>
   <si>
-    <t xml:space="preserve">Framework FACT
+    <t>Framework FACT
 (Feeling-Action-Context-Thinking)</t>
   </si>
   <si>
-    <t xml:space="preserve">✗ TIDAK ADA
+    <t>✗ TIDAK ADA
 (tidak ada di prompt evaluate lama)</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ DITAMBAHKAN — 4 dimensi skor 1-10,
+    <t>✓ DITAMBAHKAN — 4 dimensi skor 1-10,
 total max 40, per QA</t>
   </si>
   <si>
     <t>BARU ⭐</t>
   </si>
   <si>
-    <t xml:space="preserve">Kompetensi Spencer &amp; Spencer
+    <t>Kompetensi Spencer &amp; Spencer
 (1993)</t>
   </si>
   <si>
-    <t xml:space="preserve">✗ TIDAK ADA
+    <t>✗ TIDAK ADA
 (tidak ada field "competency" di schema lama)</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ DITAMBAHKAN — per QA:
+    <t>✓ DITAMBAHKAN — per QA:
 code, name, level 1-5, behavior_note
 + competency_scores rekapitulasi keseluruhan</t>
   </si>
   <si>
-    <t xml:space="preserve">Kamus Kompetensi
+    <t>Kamus Kompetensi
 (konteks file)</t>
   </si>
   <si>
-    <t xml:space="preserve">✗ TIDAK ADA
+    <t>✗ TIDAK ADA
 (tidak ada file kamus kompetensi)</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ DITAMBAHKAN
+    <t>✓ DITAMBAHKAN
 contexts/kamus-kompetensi-sp-sp.md
 (file baru, ada di baru saja)</t>
   </si>
@@ -188,22 +205,22 @@
     <t>Candidate Archetype</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ ADA — 7 tipe archetype berbasis
+    <t>✓ ADA — 7 tipe archetype berbasis
 pola ConCISE</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ ADA — 7 tipe archetype berbasis
+    <t>✓ ADA — 7 tipe archetype berbasis
 pola ConCISE (sama)</t>
   </si>
   <si>
     <t>Filler Words Analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">✗ TIDAK ADA di schema lama
+    <t>✗ TIDAK ADA di schema lama
 (tidak muncul di required fields)</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ ADA — analisis kata filler
+    <t>✓ ADA — analisis kata filler
 (dibuktikan dari unit test TC-UNIT-01 s/d 06)</t>
   </si>
   <si>
@@ -219,16 +236,16 @@
     <t>Field "recommendation_verdict"</t>
   </si>
   <si>
-    <t xml:space="preserve">Jumlah required fields
+    <t>Jumlah required fields
 per QA object</t>
   </si>
   <si>
-    <t xml:space="preserve">8 field:
+    <t>8 field:
 question, answer, star, concise,
 rating, suggestion, hack, better_answer_example</t>
   </si>
   <si>
-    <t xml:space="preserve">10 field (+2 field baru):
+    <t>10 field (+2 field baru):
 question, answer, star, FACT, competency,
 concise, rating, suggestion, hack, better_answer_example</t>
   </si>
@@ -236,14 +253,14 @@
     <t>── D. MODUL COACHING ──</t>
   </si>
   <si>
-    <t xml:space="preserve">System Prompt
+    <t>System Prompt
 Coaching Chat</t>
   </si>
   <si>
     <t>Prompt generik (tidak spesifik persona)</t>
   </si>
   <si>
-    <t xml:space="preserve">Persona eksplisit: "Siti Rahayu — HR Director 20 tahun pengalaman"
+    <t>Persona eksplisit: "Siti Rahayu — HR Director 20 tahun pengalaman"
 Mentions FACT &amp; Spencer &amp; Spencer secara eksplisit di prompt</t>
   </si>
   <si>
@@ -364,7 +381,7 @@
     <t>✗ TIDAK ADA</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ ADA — rekapitulasi kompetensi Spencer
+    <t>✓ ADA — rekapitulasi kompetensi Spencer
 per kompetensi: code, name, level, score, summary</t>
   </si>
   <si>
@@ -380,7 +397,7 @@
     <t>Output: candidate_archetype</t>
   </si>
   <si>
-    <t xml:space="preserve">PERBANDINGAN HASIL PENGUJIAN — MODEL LAMA vs MODEL BARU
+    <t>PERBANDINGAN HASIL PENGUJIAN — MODEL LAMA vs MODEL BARU
 Sumber: Hasil pengujian nyata model baru (TC-API-06) + analisis kode model lama</t>
   </si>
   <si>
@@ -390,11 +407,11 @@
     <t>Endpoint</t>
   </si>
   <si>
-    <t xml:space="preserve">Model LAMA
+    <t>Model LAMA
 (estimasi dari kode)</t>
   </si>
   <si>
-    <t xml:space="preserve">Model BARU
+    <t>Model BARU
 (data nyata dari pengujian)</t>
   </si>
   <si>
@@ -404,20 +421,20 @@
     <t>⚠️  CATATAN JUJUR: Model LAMA tidak dijalankan pengujiannya dalam sesi ini. Kolom "Model LAMA" berisi analisis kode/prompt, BUKAN hasil eksekusi nyata. Model BARU memiliki data hasil pengujian nyata (24 TC).</t>
   </si>
   <si>
-    <t xml:space="preserve">Framework Evaluasi
+    <t>Framework Evaluasi
 yang Tersedia</t>
   </si>
   <si>
     <t>/api/evaluate</t>
   </si>
   <si>
-    <t xml:space="preserve">STAR ✓
+    <t>STAR ✓
 ConCISE ✓
 FACT ✗ (tidak ada)
 Spencer &amp; Spencer ✗ (tidak ada)</t>
   </si>
   <si>
-    <t xml:space="preserve">STAR ✓
+    <t>STAR ✓
 ConCISE ✓
 FACT ✓ (ditambahkan)
 Spencer &amp; Spencer ✓ (ditambahkan)</t>
@@ -426,30 +443,30 @@
     <t>Model baru punya 4 framework vs 2 di model lama</t>
   </si>
   <si>
-    <t xml:space="preserve">Jumlah Field
+    <t>Jumlah Field
 Output per QA</t>
   </si>
   <si>
-    <t xml:space="preserve">8 required fields
+    <t>8 required fields
 (tanpa FACT &amp; competency)</t>
   </si>
   <si>
-    <t xml:space="preserve">10 required fields
+    <t>10 required fields
 (+fact, +competency)</t>
   </si>
   <si>
     <t>+2 field baru yang dibuktikan dari analisis kode</t>
   </si>
   <si>
-    <t xml:space="preserve">Hasil Pengujian
+    <t>Hasil Pengujian
 API Evaluate</t>
   </si>
   <si>
-    <t xml:space="preserve">TIDAK DIUJI dalam sesi ini
+    <t>TIDAK DIUJI dalam sesi ini
 (data kode: schema berbeda)</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-API-06: ✓ LULUS
+    <t>TC-API-06: ✓ LULUS
 Overall: 92/100
 Archetype: The Star Performer
 Avg STAR: 4.0/4
@@ -460,19 +477,19 @@
     <t>Hanya model baru yang memiliki hasil pengujian terukur</t>
   </si>
   <si>
-    <t xml:space="preserve">Hasil Pengujian
+    <t>Hasil Pengujian
 API Coaching Chat</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/coaching
+    <t>/api/coaching
 (action: chat)</t>
   </si>
   <si>
-    <t xml:space="preserve">TIDAK DIUJI
+    <t>TIDAK DIUJI
 (struktur sama, prompt berbeda)</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-API-07: ✓ LULUS
+    <t>TC-API-07: ✓ LULUS
 Respons: 1.151 chars
 Kontekstual dengan evaluasi
 Durasi: 8.007 ms</t>
@@ -481,19 +498,19 @@
     <t>Model baru punya persona Siti Rahayu yang lebih kaya</t>
   </si>
   <si>
-    <t xml:space="preserve">Hasil Pengujian
+    <t>Hasil Pengujian
 API TTS Audio</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/coaching
+    <t>/api/coaching
 (action: speech)</t>
   </si>
   <si>
-    <t xml:space="preserve">TIDAK DIUJI
+    <t>TIDAK DIUJI
 (kode identik)</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-API-08: ✓ LULUS
+    <t>TC-API-08: ✓ LULUS
 333.504 chars base64
 MIME: audio/L16;codec=pcm;rate=24000
 Durasi: 6.185 ms</t>
@@ -502,19 +519,19 @@
     <t>Kode TTS identik di kedua model</t>
   </si>
   <si>
-    <t xml:space="preserve">Hasil Pengujian
+    <t>Hasil Pengujian
 Unit Test</t>
   </si>
   <si>
-    <t xml:space="preserve">lib/evaluate.ts
+    <t>lib/evaluate.ts
 lib/audio-manager.ts</t>
   </si>
   <si>
-    <t xml:space="preserve">TIDAK DIUJI
+    <t>TIDAK DIUJI
 (70 baris vs 92 baris di baru)</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-UNIT-01 s/d 10: ✓ SEMUA LULUS
+    <t>TC-UNIT-01 s/d 10: ✓ SEMUA LULUS
 Filler: 6 TC lulus
 WAV: 2 TC lulus
 JSON: 2 TC lulus</t>
@@ -523,18 +540,18 @@
     <t>Unit test hanya dijalankan untuk model baru</t>
   </si>
   <si>
-    <t xml:space="preserve">Hasil Pengujian
+    <t>Hasil Pengujian
 E2E Playwright</t>
   </si>
   <si>
     <t>Halaman UI</t>
   </si>
   <si>
-    <t xml:space="preserve">TIDAK DIUJI
+    <t>TIDAK DIUJI
 (folder lama, server berbeda)</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-E2E-01 s/d 04: ✓ SEMUA LULUS
+    <t>TC-E2E-01 s/d 04: ✓ SEMUA LULUS
 Landing: 11.400ms
 Login: 10.857ms
 Mobile 390px: OK
@@ -544,40 +561,40 @@
     <t>E2E hanya dijalankan untuk model baru (port 3000)</t>
   </si>
   <si>
-    <t xml:space="preserve">Komponen
+    <t>Komponen
 InterviewEvaluation</t>
   </si>
   <si>
     <t>UI Component</t>
   </si>
   <si>
-    <t xml:space="preserve">2.129 baris
+    <t>2.129 baris
 (chart evaluasi, tampilan skor)</t>
   </si>
   <si>
-    <t xml:space="preserve">2.371 baris (+242 baris)
+    <t>2.371 baris (+242 baris)
 (penambahan display FACT &amp; Spencer chart)</t>
   </si>
   <si>
     <t>Model baru menampilkan lebih banyak output evaluasi</t>
   </si>
   <si>
-    <t xml:space="preserve">LiveInterview
+    <t>LiveInterview
 Component</t>
   </si>
   <si>
-    <t xml:space="preserve">1.473 baris
+    <t>1.473 baris
 (live voice session)</t>
   </si>
   <si>
-    <t xml:space="preserve">1.066 baris (-407 baris)
+    <t>1.066 baris (-407 baris)
 (refactoring, lebih ringkas)</t>
   </si>
   <si>
     <t>Model baru hasil refactoring — lebih maintainable</t>
   </si>
   <si>
-    <t xml:space="preserve">DELTA FITUR — PERUBAHAN DARI MODEL LAMA KE MODEL BARU
+    <t>DELTA FITUR — PERUBAHAN DARI MODEL LAMA KE MODEL BARU
 Berdasarkan Analisis Kode Nyata (Diff antara dua folder proyek)</t>
   </si>
   <si>
@@ -602,7 +619,7 @@
     <t>1</t>
   </si>
   <si>
-    <t xml:space="preserve">FACT Framework
+    <t>FACT Framework
 (Feeling-Action-Context-Thinking)</t>
   </si>
   <si>
@@ -621,7 +638,7 @@
     <t>2</t>
   </si>
   <si>
-    <t xml:space="preserve">Spencer &amp; Spencer (1993)
+    <t>Spencer &amp; Spencer (1993)
 Kompetensi per QA</t>
   </si>
   <si>
@@ -634,7 +651,7 @@
     <t>3</t>
   </si>
   <si>
-    <t xml:space="preserve">Kamus Kompetensi
+    <t>Kamus Kompetensi
 (contexts/kamus-kompetensi-sp-sp.md)</t>
   </si>
   <si>
@@ -653,7 +670,7 @@
     <t>4</t>
   </si>
   <si>
-    <t xml:space="preserve">Persona Coaching
+    <t>Persona Coaching
 "Siti Rahayu"</t>
   </si>
   <si>
@@ -669,7 +686,7 @@
     <t>5</t>
   </si>
   <si>
-    <t xml:space="preserve">lib/evaluate.ts
+    <t>lib/evaluate.ts
 (+22 baris, +31%)</t>
   </si>
   <si>
@@ -688,7 +705,7 @@
     <t>6</t>
   </si>
   <si>
-    <t xml:space="preserve">app/api/evaluate/route.ts
+    <t>app/api/evaluate/route.ts
 (+38 baris, +18%)</t>
   </si>
   <si>
@@ -701,7 +718,7 @@
     <t>7</t>
   </si>
   <si>
-    <t xml:space="preserve">components/InterviewEvaluation.tsx
+    <t>components/InterviewEvaluation.tsx
 (+242 baris, +11%)</t>
   </si>
   <si>
@@ -714,7 +731,7 @@
     <t>8</t>
   </si>
   <si>
-    <t xml:space="preserve">components/LiveInterview.tsx
+    <t>components/LiveInterview.tsx
 (-407 baris, -28%)</t>
   </si>
   <si>
@@ -733,7 +750,7 @@
     <t>9</t>
   </si>
   <si>
-    <t xml:space="preserve">Firebase
+    <t>Firebase
 (12.12.1 → 12.19.0)</t>
   </si>
   <si>
@@ -752,14 +769,14 @@
     <t>10</t>
   </si>
   <si>
-    <t xml:space="preserve">Required Fields
+    <t>Required Fields
 /api/evaluate per QA</t>
   </si>
   <si>
     <t>PERLUASAN SCHEMA</t>
   </si>
   <si>
-    <t xml:space="preserve">Lama: 8 fields [question, answer, star, concise, rating, suggestion, hack, better_answer_example]
+    <t>Lama: 8 fields [question, answer, star, concise, rating, suggestion, hack, better_answer_example]
 Baru: 10 fields [+fact, +competency]</t>
   </si>
   <si>
@@ -775,7 +792,7 @@
     <t>Perbedaan Paling Signifikan</t>
   </si>
   <si>
-    <t xml:space="preserve">Model BARU menambahkan 2 framework evaluasi baru yang TIDAK ADA di model lama:
+    <t>Model BARU menambahkan 2 framework evaluasi baru yang TIDAK ADA di model lama:
 (1) FACT Framework (Feeling/Action/Context/Thinking) — 4 dimensi skor /10 per QA
 (2) Spencer &amp; Spencer (1993) Competency Assessment — level 1-5 per kompetensi per QA
 Ini adalah perubahan substansial pada engine evaluasi inti sistem.</t>
@@ -784,28 +801,28 @@
     <t>Jumlah Framework Evaluasi</t>
   </si>
   <si>
-    <t xml:space="preserve">Model LAMA: 2 framework (STAR + ConCISE)
+    <t>Model LAMA: 2 framework (STAR + ConCISE)
 Model BARU: 4 framework (STAR + ConCISE + FACT + Spencer &amp; Spencer)</t>
   </si>
   <si>
     <t>Jumlah Field Output per QA</t>
   </si>
   <si>
-    <t xml:space="preserve">Model LAMA: 8 required fields
+    <t>Model LAMA: 8 required fields
 Model BARU: 10 required fields (+fact, +competency)</t>
   </si>
   <si>
     <t>Ketersediaan Kamus Referensi</t>
   </si>
   <si>
-    <t xml:space="preserve">Model LAMA: Tidak ada file kamus kompetensi
+    <t>Model LAMA: Tidak ada file kamus kompetensi
 Model BARU: Ada contexts/kamus-kompetensi-sp-sp.md sebagai ground-truth Spencer &amp; Spencer</t>
   </si>
   <si>
     <t>Perubahan Komponen Terbesar</t>
   </si>
   <si>
-    <t xml:space="preserve">LiveInterview.tsx: -407 baris (refactoring besar, kode lebih ringkas)
+    <t>LiveInterview.tsx: -407 baris (refactoring besar, kode lebih ringkas)
 InterviewEvaluation.tsx: +242 baris (visualisasi baru untuk FACT &amp; Spencer)</t>
   </si>
   <si>
@@ -830,7 +847,7 @@
     <t>Untuk Kelas TA Besok</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Tunjukkan tabel ini sebagai bukti perbedaan framework: Model Lama (2 framework) vs Model Baru (4 framework)
+    <t>1. Tunjukkan tabel ini sebagai bukti perbedaan framework: Model Lama (2 framework) vs Model Baru (4 framework)
 2. Jelaskan bahwa penambahan FACT dan Spencer &amp; Spencer adalah kontribusi utama model baru
 3. Siapkan demo langsung sistem baru untuk menunjukkan output dengan 4 framework sekaligus</t>
   </si>
@@ -838,7 +855,7 @@
     <t>Untuk Kesempurnaan Data</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Jalankan skenario pengujian yang sama di model lama (jika server bisa dijalankan)
+    <t>1. Jalankan skenario pengujian yang sama di model lama (jika server bisa dijalankan)
 2. Bandingkan output JSON /api/evaluate secara numerik (skor, field yang tersedia)
 3. Dokumentasikan sebagai tabel perbandingan kuantitatif untuk BAB IV skripsi</t>
   </si>
@@ -846,98 +863,98 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="16" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
+      <color rgb="FF212121"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1A237E"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1B5E20"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF6C757D"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF212121"/>
       <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF1A237E"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF1B5E20"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF6C757D"/>
-      <sz val="10"/>
+      <color rgb="FF0C5460"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF0C5460"/>
       <sz val="10"/>
+      <color rgb="FF1B5E20"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1B5E20"/>
-      <sz val="10"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
+      <sz val="10"/>
+      <color rgb="FF856404"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF856404"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF212121"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF856404"/>
       <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF856404"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF212121"/>
-      <sz val="10"/>
+      <color rgb="FF721C24"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF721C24"/>
       <sz val="10"/>
+      <color rgb="FF6C757D"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF6C757D"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="13"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1023,10 +1040,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1048,97 +1073,100 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1478,9 +1506,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:E49"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -1488,656 +1516,656 @@
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="50" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="2:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:5" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+    </row>
+    <row r="3" spans="2:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+    </row>
+    <row r="5" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="9" t="s">
+    <row r="6" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="5" t="s">
+    <row r="7" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="9" t="s">
+    <row r="8" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
+    <row r="9" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="9" t="s">
+    <row r="10" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="5" t="s">
+    <row r="11" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="2" t="s">
+    <row r="12" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+    </row>
+    <row r="13" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="9" t="s">
+    <row r="14" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="5" t="s">
+    <row r="15" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="9" t="s">
+    <row r="16" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
+    <row r="17" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+    </row>
+    <row r="18" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="5" t="s">
+    <row r="19" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20" s="9" t="s">
+    <row r="20" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="5" t="s">
+    <row r="21" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="9" t="s">
+    <row r="22" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B23" s="5" t="s">
+    <row r="23" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B24" s="9" t="s">
+    <row r="24" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="5" t="s">
+    <row r="25" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B26" s="9" t="s">
+    <row r="26" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="27" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="5" t="s">
+    <row r="27" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="2" t="s">
+    <row r="28" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" s="5" t="s">
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+    </row>
+    <row r="29" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E29" s="11" t="s">
+      <c r="E29" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="30" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30" s="9" t="s">
+    <row r="30" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31" s="5" t="s">
+    <row r="31" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="32" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="9" t="s">
+    <row r="32" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="E32" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="33" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="5" t="s">
+    <row r="33" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" s="2" t="s">
+    <row r="34" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-    </row>
-    <row r="35" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="5" t="s">
+      <c r="C34" s="27"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+    </row>
+    <row r="35" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B36" s="9" t="s">
+    <row r="36" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="37" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B37" s="5" t="s">
+    <row r="37" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="38" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B38" s="9" t="s">
+    <row r="38" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="39" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B39" s="5" t="s">
+    <row r="39" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="40" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B40" s="9" t="s">
+    <row r="40" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="E40" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="41" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B41" s="5" t="s">
+    <row r="41" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="E41" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="42" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B42" s="9" t="s">
+    <row r="42" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="43" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B43" s="5" t="s">
+    <row r="43" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E43" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B44" s="2" t="s">
+    <row r="44" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-    </row>
-    <row r="45" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B45" s="5" t="s">
+      <c r="C44" s="27"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+    </row>
+    <row r="45" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D45" s="7" t="s">
+      <c r="D45" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="E45" s="11" t="s">
+      <c r="E45" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="46" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B46" s="9" t="s">
+    <row r="46" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E46" s="11" t="s">
+      <c r="E46" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="47" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B47" s="5" t="s">
+    <row r="47" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D47" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E47" s="8" t="s">
+      <c r="E47" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="48" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B48" s="9" t="s">
+    <row r="48" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="7" t="s">
+      <c r="D48" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="E48" s="8" t="s">
+      <c r="E48" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="49" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B49" s="5" t="s">
+    <row r="49" spans="2:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D49" s="7" t="s">
+      <c r="D49" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E49" s="8" t="s">
+      <c r="E49" s="7" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B44:E44"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B44:E44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:F14"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -2146,192 +2174,192 @@
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="40" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="2:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-    </row>
-    <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="26" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="2:6" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="2:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="13" t="s">
+    <row r="5" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-    </row>
-    <row r="6" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+    </row>
+    <row r="6" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="12" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="9" t="s">
+    <row r="7" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="12" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="5" t="s">
+    <row r="8" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="9" t="s">
+    <row r="9" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="12" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
+    <row r="10" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="12" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="5" t="s">
+    <row r="12" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="12" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="9" t="s">
+    <row r="13" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="12" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="5" t="s">
+    <row r="14" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="12" t="s">
         <v>157</v>
       </c>
     </row>
@@ -2341,14 +2369,14 @@
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:G14"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2359,233 +2387,233 @@
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="36" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="16" t="s">
+    <row r="2" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="17" t="s">
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="4" spans="2:7" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="18" t="s">
+    <row r="5" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="16" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="21" t="s">
+    <row r="6" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="16" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="7" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="18" t="s">
+    <row r="7" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="19" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="8" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="21" t="s">
+    <row r="8" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="G8" s="19" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="9" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="18" t="s">
+    <row r="9" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="20" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="10" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="21" t="s">
+    <row r="10" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="20" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="11" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="18" t="s">
+    <row r="11" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="20" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="12" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="21" t="s">
+    <row r="12" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="G12" s="24" t="s">
+      <c r="G12" s="20" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="13" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
+    <row r="13" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="G13" s="24" t="s">
+      <c r="G13" s="20" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="14" ht="70" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="21" t="s">
+    <row r="14" spans="2:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="20" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2594,113 +2622,113 @@
     <mergeCell ref="B2:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:C15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="65" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="26" t="s">
+    <row r="2" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="31" t="s">
         <v>217</v>
       </c>
-      <c r="C2" s="26"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
+      <c r="C2" s="31"/>
+    </row>
+    <row r="4" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+      <c r="C4" s="27"/>
+    </row>
+    <row r="5" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="15" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
+    <row r="6" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="15" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="7" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="5" t="s">
+    <row r="7" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="15" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="8" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="5" t="s">
+    <row r="8" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="15" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="9" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
+    <row r="9" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="15" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="2" t="s">
+    <row r="10" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="27" t="s">
         <v>229</v>
       </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="27" t="s">
+      <c r="C10" s="27"/>
+    </row>
+    <row r="11" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="23" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="12" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="27" t="s">
+    <row r="12" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="23" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
+    <row r="13" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="27" t="s">
         <v>234</v>
       </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="29" t="s">
+      <c r="C13" s="27"/>
+    </row>
+    <row r="14" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="25" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="15" ht="55" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="29" t="s">
+    <row r="15" spans="2:3" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="25" t="s">
         <v>238</v>
       </c>
     </row>
@@ -2712,6 +2740,6 @@
     <mergeCell ref="B13:C13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>